<commit_message>
feat(agents): increase max output tokens and enhance caching with verification callbacks
- Increase max_output_tokens to 65535 across all analytics agent models for better content generation
- Add comprehensive logging to marking scheme cache callbacks with agent name context
- Implement error handling for JSON parsing failures in cache operations
- Add validation checks for questions data before caching
- Create new marking_scheme_verification_cache_callbacks function for final output caching
- Improve cache callback robustness with detailed error tracking and logging
- Update sample marking scheme files with verification documentation
- Enhance before_callback to properly handle cached responses without triggering Vertex AI processing
- Add detailed logging at info level for cache hits, misses, and error conditions
</commit_message>
<xml_diff>
--- a/sample/VTC Test Marking Scheme.xlsx
+++ b/sample/VTC Test Marking Scheme.xlsx
@@ -462,15 +462,25 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>The Role of VTC. The VTC is the largest provider of VPET in Hong Kong. Briefly explain what VPET stands for and why it is important for Hong Kong’s workforce development.</t>
+          <t>The Role of VTC: The VTC is the largest provider of VPET in Hong Kong. Briefly explain what VPET stands for and why it is important for Hong Kong’s workforce development.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>- Correctly stating **Vocational and Professional Education and Training** (2 marks)  - Explaining focus on **practical skills** or **specialized trades** (4 marks)  - Explaining benefit to the workforce such as **reducing skills gap** or **employment readiness** (4 marks)
+          <t>- Correctly stating "**Vocational and Professional Education and Training**" (2 marks)
+- Explaining focus on **practical skills** or **specialized trades** (4 marks)
+- Explaining benefit to workforce (reducing skills gap, employment readiness) (4 marks)
+**General Grading Principles:**
+- **9-10 marks**: Complete, accurate, correct terminology, and well-explained.
+- **6-8 marks**: Mostly correct but misses a specific detail or vague explanation.
+- **3-5 marks**: Basic understanding but misses core point.
+- **0-2 marks**: Incorrect or irrelevant.
 ---
 **General Grading Guide:**
-- **9-10 marks**: The answer is complete, accurate, uses correct terminology, and is well-explained.  - **6-8 marks**: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague.  - **3-5 marks**: The student shows basic understanding but misses the core point or only answers half the question.  - **0-2 marks**: The answer is largely incorrect, irrelevant, or blank.</t>
+- **9-10 marks**: The answer is complete, accurate, uses correct terminology, and is well-explained.
+- **6-8 marks**: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague.
+- **3-5 marks**: The student shows basic understanding but misses the core point or only answers half the question.
+- **0-2 marks**: The answer is largely incorrect, irrelevant, or blank.</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -485,15 +495,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Member Institutions. Compare IVE (Hong Kong Institute of Vocational Education) and THEi (Technological and Higher Education Institute of Hong Kong). What is the main difference between the types of qualifications/programmes offered by these two institutions?</t>
+          <t>Member Institutions: Compare IVE (Hong Kong Institute of Vocational Education) and THEi (Technological and Higher Education Institute of Hong Kong). What is the main difference between the types of qualifications/programmes offered by these two institutions?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>- Correctly identifying that **IVE** primarily focuses on **Higher Diploma (HD)** programmes / technical training (5 marks)  - Correctly identifying that **THEi** focuses on vocationally-oriented **Bachelor’s Degree** programmes (5 marks)
+          <t>- Correctly identifying that **IVE** primarily focuses on **Higher Diploma (HD)** programmes (5 marks)
+- Correctly identifying that **THEi** focuses on vocationally-oriented **Bachelor’s Degree** programmes (5 marks)
+**General Grading Principles:**
+- **9-10 marks**: Complete, accurate, correct terminology, and well-explained.
+- **6-8 marks**: Mostly correct but misses a specific detail or vague explanation.
+- **3-5 marks**: Basic understanding but misses core point.
+- **0-2 marks**: Incorrect or irrelevant.
 ---
 **General Grading Guide:**
-- **9-10 marks**: The answer is complete, accurate, uses correct terminology, and is well-explained.  - **6-8 marks**: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague.  - **3-5 marks**: The student shows basic understanding but misses the core point or only answers half the question.  - **0-2 marks**: The answer is largely incorrect, irrelevant, or blank.</t>
+- **9-10 marks**: The answer is complete, accurate, uses correct terminology, and is well-explained.
+- **6-8 marks**: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague.
+- **3-5 marks**: The student shows basic understanding but misses the core point or only answers half the question.
+- **0-2 marks**: The answer is largely incorrect, irrelevant, or blank.</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -508,15 +527,25 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Educational Philosophy. VTC emphasizes the "Think and Do" approach. Explain what this phrase means in the context of a student's learning experience.</t>
+          <t>Educational Philosophy: VTC emphasizes the " Think and Do" approach. Explain what this phrase means in the context of a student's learning experience.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>- Explaining **"Think"** as theory or academic knowledge (3 marks)  - Explaining **"Do"** as practical skills or hands-on application (3 marks)  - Explaining the **synthesis**: solving problems by combining both head and hands (4 marks)
+          <t>- Explaining "**Think**" (Theory/Academic knowledge) (3 marks)
+- Explaining "**Do**" (Practical skills/Hands-on) (3 marks)
+- Explaining the **synthesis**: Being able to solve problems by combining both head and hands (4 marks)
+**General Grading Principles:**
+- **9-10 marks**: Complete, accurate, correct terminology, and well-explained.
+- **6-8 marks**: Mostly correct but misses a specific detail or vague explanation.
+- **3-5 marks**: Basic understanding but misses core point.
+- **0-2 marks**: Incorrect or irrelevant.
 ---
 **General Grading Guide:**
-- **9-10 marks**: The answer is complete, accurate, uses correct terminology, and is well-explained.  - **6-8 marks**: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague.  - **3-5 marks**: The student shows basic understanding but misses the core point or only answers half the question.  - **0-2 marks**: The answer is largely incorrect, irrelevant, or blank.</t>
+- **9-10 marks**: The answer is complete, accurate, uses correct terminology, and is well-explained.
+- **6-8 marks**: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague.
+- **3-5 marks**: The student shows basic understanding but misses the core point or only answers half the question.
+- **0-2 marks**: The answer is largely incorrect, irrelevant, or blank.</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -531,15 +560,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Study Pathways. If a Secondary 6 student does not achieve the minimum entrance requirements for a Bachelor's Degree or a Higher Diploma, what is the VTC study pathway available to them to eventually reach a Higher Diploma level? (Name the specific foundation programme).</t>
+          <t>Study Pathways: If a Secondary 6 student does not achieve the minimum entrance requirements for a Bachelor's Degree or a Higher Diploma, what is the VTC study pathway available to them to eventually reach a Higher Diploma level? (Name the specific foundation programme).</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>- Correctly naming the **Diploma of Foundation Studies (DFS)** or **Diploma of Vocational Education (DVE)** (5 marks)  - Explanation of the **progression**: completion of the diploma allows entry to VTC **Higher Diploma (HD)** programmes (5 marks)
+          <t>- Correctly naming the "**Diploma of Foundation Studies**" (DFS) or "**Diploma of Vocational Education**" (DVE) (5 marks)
+- Explanation of the **progression** (Completion of DFS allows entry to Higher Diploma) (5 marks)
+**General Grading Principles:**
+- **9-10 marks**: Complete, accurate, correct terminology, and well-explained.
+- **6-8 marks**: Mostly correct but misses a specific detail or vague explanation.
+- **3-5 marks**: Basic understanding but misses core point.
+- **0-2 marks**: Incorrect or irrelevant.
 ---
 **General Grading Guide:**
-- **9-10 marks**: The answer is complete, accurate, uses correct terminology, and is well-explained.  - **6-8 marks**: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague.  - **3-5 marks**: The student shows basic understanding but misses the core point or only answers half the question.  - **0-2 marks**: The answer is largely incorrect, irrelevant, or blank.</t>
+- **9-10 marks**: The answer is complete, accurate, uses correct terminology, and is well-explained.
+- **6-8 marks**: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague.
+- **3-5 marks**: The student shows basic understanding but misses the core point or only answers half the question.
+- **0-2 marks**: The answer is largely incorrect, irrelevant, or blank.</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -554,15 +592,25 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Industry Partnership. Why does the VTC collaborate closely with industry partners (companies and trade associations)? Give two examples of how this benefits students.</t>
+          <t>Industry Partnership: Why does the VTC collaborate closely with industry partners (companies and trade associations)? Give two examples of how this benefits students.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>- General explanation regarding **curriculum relevance** or meeting **industry needs** (4 marks)  - **First specific benefit**: e.g., Internships or work-integrated learning (3 marks)  - **Second specific benefit**: e.g., Job placement support or access to industry-standard equipment (3 marks)
+          <t>- **General explanation**: Ensuring curriculum is up-to-date with market trends/industry needs (4 marks)
+- **First specific benefit**: e.g., Internship/Work-integrated learning opportunities (3 marks)
+- **Second specific benefit**: e.g., Job placement support or access to industry-standard equipment (3 marks)
+**General Grading Principles:**
+- **9-10 marks**: Complete, accurate, correct terminology, and well-explained.
+- **6-8 marks**: Mostly correct but misses a specific detail or vague explanation.
+- **3-5 marks**: Basic understanding but misses core point.
+- **0-2 marks**: Incorrect or irrelevant.
 ---
 **General Grading Guide:**
-- **9-10 marks**: The answer is complete, accurate, uses correct terminology, and is well-explained.  - **6-8 marks**: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague.  - **3-5 marks**: The student shows basic understanding but misses the core point or only answers half the question.  - **0-2 marks**: The answer is largely incorrect, irrelevant, or blank.</t>
+- **9-10 marks**: The answer is complete, accurate, uses correct terminology, and is well-explained.
+- **6-8 marks**: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague.
+- **3-5 marks**: The student shows basic understanding but misses the core point or only answers half the question.
+- **0-2 marks**: The answer is largely incorrect, irrelevant, or blank.</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -655,7 +703,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>The marking scheme is highly reliable. It uses the correct institutional names, follows the current Hong Kong education framework (HKQF), and accurately reflects VTC’s specific branding (e.g., "Think and Do"). Final Recommendation: The scheme is ready for use. No major changes are required. Citations: [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFZzN6mUhSLE_Cle6Th_ponMGy2YTfJQMWjlaDUdb-zd2N_M1YZsBYEtNv6V5Z-o1zEwX3MB4kgw6lvZfNkiuN6Nsl9zONnR7ecV5NHkWTGf06aC1XssqlAXyA94KILl9xpNAt3gdtRLDy9BbOmgs7kmJfJBvrhTJnuZy8ZJxKxpUz0ShTiCXnOr4EYaG4=) [youtube.com](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEY46mKgA56eLWSmsyghYKTr9TI1Jxtoz8C_fqUfVePcHMNJpqj9kwcQfyrdBOmw1a_re4a4BB9dfnwx3Ixw8uDe1WDzGFHePfBPAghqf-BUoKhD8aFz6dcWlPNhL0LWWqK9NwPI-Y=)</t>
+          <t>The marking scheme is highly reliable and ready for use. The grading principles are standard and provide clear guidance for examiners. No major factual corrections are required. Citations: [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQElJ6ae_XX1fSF4qAd_yQA0pHnvM38WYAhlD9FcBoidPrMwTnoDHXiVdJU3RfGAN2QFMFtlCtDjSbSIiQTMRe25FfdNaSvLDPsQkR_zLISO6CUQvr8jl4BSpiUu_I3OHLmv0hBS7p5X), [iabhongkong.com](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFPIVY4XTJqLnRvOU3LxfjLPt3iOK6FJ1b__xoGSq88VKE65cFg_K8QKfbS_r35lwrdW3ksMrGw44EDsXMdaYipcWrW7r-5Ogd4_gCuw-LqyUXLTrVufc3Gm5pt8vUqvRfBInA=), [vpet.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFM6tvSdmxdKA3yqUoNlOCR9WBTnj0lsvVHqFe8wU9lqrFTP1fj17oNFPzYXbtwohZDlrcWXJhRLxGEKOhUeNG56R8SPlIUNInrevOwgRKou8XNqqN5HF5B-Cth3TOOUhXf574SDjyuHw==), [ive.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGVPjHvdEClJO6ukbafrBmZPdL9ZeUXyzvHdMZN0_hX5Rhl8AKPbToO6aqdxp-a4UTXIDhggR-EaQc_ZN7g2Mj0HwImZZ3achzmXcAcK1NRLUwd-Yo=), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH0X_eh7ezfDsytvWaPpj3fugqSBmhzHI8Pvh9IBWEZLV2Z2Y_2kqaTFrlkcbEVNj2yi292roCsBLzvO4LjPugEvU4apVaVqP0TY7Fe2QHSM30PJ8H-2-j-4Vf4myspXphg8dqPMEp6LEDhR92EHyMcnaQle84jZAEMO98s1A==), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEuElx1sGvFCohYYBaWDF7ImlaXk0hPbElbF1WLOU3ipgox4NI5CRK5v-tqdkFJOqQoKwCgIXWjGnFbk1UXhYWTRrFboZRsdwxbln1F_HtwWPVTq-NjIrIPqu4h4qPgcceeqkrCOnMKZqDOY9CXUgkpuBvWHA==)</t>
         </is>
       </c>
     </row>
@@ -667,7 +715,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-01-09 07:26:58</t>
+          <t>2026-01-17 11:40:49</t>
         </is>
       </c>
     </row>
@@ -734,7 +782,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>The Role of VTC. The VTC is the largest provider of VPET in Hong Kong. Briefly explain what VPET stands for and why it is important for Hong Kong’s workforce development.</t>
+          <t>The Role of VTC: The VTC is the largest provider of VPET in Hong Kong. Briefly explain what VPET stands for and why it is important for Hong Kong’s workforce development.</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -749,7 +797,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Member Institutions. Compare IVE (Hong Kong Institute of Vocational Education) and THEi (Technological and Higher Education Institute of Hong Kong). What is the main difference between the types of qualifications/programmes offered by these two institutions?</t>
+          <t>Member Institutions: Compare IVE (Hong Kong Institute of Vocational Education) and THEi (Technological and Higher Education Institute of Hong Kong). What is the main difference between the types of qualifications/programmes offered by these two institutions?</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -764,7 +812,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Educational Philosophy. VTC emphasizes the "Think and Do" approach. Explain what this phrase means in the context of a student's learning experience.</t>
+          <t>Educational Philosophy: VTC emphasizes the " Think and Do" approach. Explain what this phrase means in the context of a student's learning experience.</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -779,7 +827,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Study Pathways. If a Secondary 6 student does not achieve the minimum entrance requirements for a Bachelor's Degree or a Higher Diploma, what is the VTC study pathway available to them to eventually reach a Higher Diploma level? (Name the specific foundation programme).</t>
+          <t>Study Pathways: If a Secondary 6 student does not achieve the minimum entrance requirements for a Bachelor's Degree or a Higher Diploma, what is the VTC study pathway available to them to eventually reach a Higher Diploma level? (Name the specific foundation programme).</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -794,7 +842,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Industry Partnership. Why does the VTC collaborate closely with industry partners (companies and trade associations)? Give two examples of how this benefits students.</t>
+          <t>Industry Partnership: Why does the VTC collaborate closely with industry partners (companies and trade associations)? Give two examples of how this benefits students.</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -934,12 +982,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>VTC is officially recognized as the largest provider of Vocational and Professional Education and Training (VPET) in Hong Kong. The acronym was updated by the Hong Kong government from "VET" to "VPET" several years ago to emphasize the "Professional" aspect. The marking points for "practical skills" and "reducing skills gap" are standard industry-aligned objectives for VTC.</t>
+          <t>VPET stands for Vocational and Professional Education and Training. VTC is officially recognized as the largest provider of VPET in Hong Kong, serving approximately 200,000 students annually. The marking points correctly identify the dual focus on practical skills and workforce development.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>You might add a note that VPET is a key pillar of Hong Kong's dual-track education system (academic vs. vocational).</t>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -954,12 +1002,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>IVE (Hong Kong Institute of Vocational Education) is the primary provider of Higher Diplomas (HD) and Foundation Diplomas. THEi (Technological and Higher Education Institute of Hong Kong) was specifically established to offer vocationally-oriented Bachelor’s Degrees. The distinction is clear and accurate. THEi degrees are often "applied" in nature, distinguishing them from traditional research-based universities.</t>
+          <t>IVE is the primary provider of Higher Diplomas (HD), while THEi was established to offer vocationally-oriented Bachelor’s Degrees. The distinction is factually sound.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mention that THEi is a "University of Applied Sciences" (UAS) candidate/member, as this is a current strategic focus for the institution.</t>
+          <t>Consider adding "Top-up Degrees" as a THEi feature for IVE Higher Diploma graduates to highlight the articulation pathway.</t>
         </is>
       </c>
     </row>
@@ -974,12 +1022,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>"Think and Do" is the official motto/approach of the VTC. It is used across their marketing and pedagogical frameworks to describe the integration of theoretical knowledge (Think) with practical application (Do). The synthesis point (4 marks) is excellent as it rewards students who understand that the two are not separate but integrated.</t>
+          <t>VTC’s official motto is "Think and Do," emphasizing the integration of theoretical knowledge with practical application. The marking scheme correctly identifies the synthesis of these elements.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>The wording is fine, but you could explicitly mention "Work-Integrated Learning" (WIL) as a specific way they implement the "Do" part.</t>
+          <t>Use the term "Applied Learning" in the marking notes, as this is the formal pedagogical term used by the Hong Kong Education Bureau (EDB).</t>
         </is>
       </c>
     </row>
@@ -994,12 +1042,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>For Secondary 6 (S6) students who do not meet the "3322+2" (Degree) or "22222" (HD) HKDSE requirements, the Diploma of Foundation Studies (DFS) is the standard one-year progression route. The Diploma of Vocational Education (DVE), offered by Youth College (a VTC member), is also a valid pathway for S6 leavers. The progression to Higher Diploma is a "through-train" approach, which is a core selling point for VTC.</t>
+          <t>For S6 students not meeting HKDSE requirements, DFS and DVE are the standard VTC entry points. The progression from DFS/DVE to Higher Diploma is a well-established pathway.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ensure the answer key accepts "Diploma of Applied Education (DAE)" as well, as it is the government-wide equivalent to the DFS/DVE, though DFS is the specific VTC-branded version.</t>
+          <t>Note that DFS is generally the more common academic foundation for S6 students aiming for IVE Higher Diplomas, whereas DVE often has a stronger focus on specific trades.</t>
         </is>
       </c>
     </row>
@@ -1014,12 +1062,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>VTC operates 25 Training Boards that include industry leaders to ensure curriculum relevance. The examples provided (internships, industry-standard equipment) are the most prominent benefits cited in VTC annual reports.</t>
+          <t>VTC maintains over 25 Training Boards and collaborates with industry partners. The benefits listed (internships, equipment, job placement) are the pillars of VTC’s industry collaboration strategy.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Another strong example is the "Earn &amp; Learn" Scheme, which allows students to work and study simultaneously with a guaranteed salary and subsidy.</t>
+          <t>Use the specific VTC terminology "Work-integrated Learning" (WIL) or "Industrial Attachment" for the internship point.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(config): centralize configuration management with config.yaml
- Add config.yaml for centralized non-sensitive configuration management
- Create config_loader.py to load and parse YAML configuration files
- Add setup_config.py and setup_config.sh scripts for automated configuration setup
- Add test_config.py to verify configuration validity and completeness
- Add docs/CONFIGURATION.md with comprehensive configuration guide
- Add docs/DOCUMENTATION_STRUCTURE.md documenting the new docs organization
- Simplify .env.template to only require API key, move all other settings to config.yaml
- Update README.md with new configuration setup instructions and quick links
- Remove obsolete documentation files (LOG_LEVEL_REVIEW_COMPLETE.md, MODEL_CONFIG_CHANGES.md)
- Update agent configuration loading to use new config.yaml structure
- Consolidate logging, caching, and model configuration into single YAML file for easier management
</commit_message>
<xml_diff>
--- a/sample/VTC Test Marking Scheme.xlsx
+++ b/sample/VTC Test Marking Scheme.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>The marking scheme is highly reliable and ready for use. The grading principles are standard and provide clear guidance for examiners. No major factual corrections are required. Citations: [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQElJ6ae_XX1fSF4qAd_yQA0pHnvM38WYAhlD9FcBoidPrMwTnoDHXiVdJU3RfGAN2QFMFtlCtDjSbSIiQTMRe25FfdNaSvLDPsQkR_zLISO6CUQvr8jl4BSpiUu_I3OHLmv0hBS7p5X), [iabhongkong.com](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFPIVY4XTJqLnRvOU3LxfjLPt3iOK6FJ1b__xoGSq88VKE65cFg_K8QKfbS_r35lwrdW3ksMrGw44EDsXMdaYipcWrW7r-5Ogd4_gCuw-LqyUXLTrVufc3Gm5pt8vUqvRfBInA=), [vpet.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFM6tvSdmxdKA3yqUoNlOCR9WBTnj0lsvVHqFe8wU9lqrFTP1fj17oNFPzYXbtwohZDlrcWXJhRLxGEKOhUeNG56R8SPlIUNInrevOwgRKou8XNqqN5HF5B-Cth3TOOUhXf574SDjyuHw==), [ive.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGVPjHvdEClJO6ukbafrBmZPdL9ZeUXyzvHdMZN0_hX5Rhl8AKPbToO6aqdxp-a4UTXIDhggR-EaQc_ZN7g2Mj0HwImZZ3achzmXcAcK1NRLUwd-Yo=), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH0X_eh7ezfDsytvWaPpj3fugqSBmhzHI8Pvh9IBWEZLV2Z2Y_2kqaTFrlkcbEVNj2yi292roCsBLzvO4LjPugEvU4apVaVqP0TY7Fe2QHSM30PJ8H-2-j-4Vf4myspXphg8dqPMEp6LEDhR92EHyMcnaQle84jZAEMO98s1A==), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEuElx1sGvFCohYYBaWDF7ImlaXk0hPbElbF1WLOU3ipgox4NI5CRK5v-tqdkFJOqQoKwCgIXWjGnFbk1UXhYWTRrFboZRsdwxbln1F_HtwWPVTq-NjIrIPqu4h4qPgcceeqkrCOnMKZqDOY9CXUgkpuBvWHA==)</t>
+          <t>This evaluation confirms that the marking scheme is factually accurate and aligns with the official standards and terminology of the Vocational Training Council (VTC) in Hong Kong. Constructive Feedback &amp; Suggestions: 1. Terminology Consistency: The marking scheme uses "Vocational and Professional Education and Training." Ensure that students are not penalized if they use the older term "Vocational Education and Training (VET)," though they should be encouraged to use the full "VPET" for full marks. 2. Grading Guide Clarity: The "General Grading Guide" is repeated multiple times in your document. You only need to state it once at the beginning or end to keep the scheme concise. 3. Qualification Levels: For Q4, it might be helpful to specify that these programmes are at QF Level 3, which allows progression to QF Level 4 (Higher Diploma). This shows a deeper understanding of the Hong Kong Qualifications Framework. Overall Verdict: The marking scheme is highly accurate and ready for use. Citations: [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHdrenv21lbr6yAbKortDcisxfdZFHSlrRnEv9gUneUBMSVzTEWl6XKekV6S7MbYYoBK09-ojdryUxmGGmiHnOT6JaEo-qv000s84W-lBTJiLtDsjGANGt6KzI=), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEiJFve_NPta3q44d6xbREsqbQPsx67t0cZtWXrVYQ-uc6To6BhcKyerxuOSxoHl-fyYG22s-zQIiDHRBqUFnY0_4POv-jjlgvjnf10SgIgasfDZJ5pnrgMXpVXUg==), [vpet.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEIUyTUeZEiL6tNf1Ez8QHkcnLOJ31pG8AqMfDijk_ZMPOwV7wHSzz3caNYHUlQHN3alPkUJVgHLoat43rwokDL0KtVng4iLYIZ2HtJGNVdhYdJM7vylk-U11mBHaLV19h1mOWg3_OdeKZH0aBH), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF1rvYIip6moTtkuw7NtxkC8p66E8wEFQBFHPMsM9pRJShxThnV5fJTc8qoGCMji8JjIbonCwUYOozutyuBmIWoVSqc-98GjUqpHgFu-ER3xtoFoveWyv7RR0od2ve7FuyzTskMeSSKtmr65DQpZyCh20vw1GcXz7z1Idtws6gqDoXhEA==), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF-a-VZrONAx6NwCVnQmgL1op0gzASrbU2LD4tGG6guQEf0PKD7Cks7RvkR1dGbXPyNGxAN2WjhQDDzZlxEz-epBbTLRZuYP-rM9UapMXjKMe6_TTXeWKqikEqWekvatU9Idv2GSsJEHSMCoBc0j_YuAw9i9y4s580M), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFBOG3zXuGfZ38LyLLgWtopL0-u8kKp5sfFkKG04DuH-z3cZoF7MvsxkxzD1SixgIlwx70hmHjkrY06t9WRD30NG_X-qx2Z1MIi9Gpoegfez2BJysy6to2QD1ALDzWxTMvYI4XlIrhYAKCgwQ9uN8e5FXEKCilmHC6usIkOngyjVNQ9)</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-01-17 11:40:49</t>
+          <t>2026-01-17 18:59:12</t>
         </is>
       </c>
     </row>
@@ -982,12 +982,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>VPET stands for Vocational and Professional Education and Training. VTC is officially recognized as the largest provider of VPET in Hong Kong, serving approximately 200,000 students annually. The marking points correctly identify the dual focus on practical skills and workforce development.</t>
+          <t>Fact Check: VPET does indeed stand for Vocational and Professional Education and Training. The VTC is the statutory body and the largest provider of VPET in Hong Kong. Answer Key Accuracy: Correct. The emphasis on practical skills and workforce development (reducing the skills gap) is the core mission of VPET as defined by the Hong Kong Education Bureau.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>You might consider adding a point for mentioning that VPET provides a "parallel pathway" to traditional academic education, as this is a key part of the government's current promotion of the sector.</t>
         </is>
       </c>
     </row>
@@ -1002,12 +1002,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>IVE is the primary provider of Higher Diplomas (HD), while THEi was established to offer vocationally-oriented Bachelor’s Degrees. The distinction is factually sound.</t>
+          <t>Fact Check: IVE (Hong Kong Institute of Vocational Education) is the primary provider of Higher Diploma (HD) and Diploma programmes. THEi (Technological and Higher Education Institute of Hong Kong) was specifically established to offer vocationally-oriented Bachelor’s Degree programmes. Answer Key Accuracy: Correct.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Consider adding "Top-up Degrees" as a THEi feature for IVE Higher Diploma graduates to highlight the articulation pathway.</t>
+          <t>To be even more precise, you could mention that THEi degrees are "Applied Degrees," which distinguishes them from traditional research-based degrees at other universities.</t>
         </is>
       </c>
     </row>
@@ -1022,12 +1022,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>VTC’s official motto is "Think and Do," emphasizing the integration of theoretical knowledge with practical application. The marking scheme correctly identifies the synthesis of these elements.</t>
+          <t>Fact Check: The "Think and Do" approach is the official motto and educational philosophy of the VTC. It is often described in official literature as "hands-on and minds-on." Answer Key Accuracy: Correct. The breakdown of "Think" (theory) and "Do" (practice) is the standard interpretation.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Use the term "Applied Learning" in the marking notes, as this is the formal pedagogical term used by the Hong Kong Education Bureau (EDB).</t>
+          <t>The marking scheme is solid. You could award bonus marks if a student mentions "problem-solving in real-world contexts," as this is a specific outcome VTC highlights for this approach.</t>
         </is>
       </c>
     </row>
@@ -1042,12 +1042,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>For S6 students not meeting HKDSE requirements, DFS and DVE are the standard VTC entry points. The progression from DFS/DVE to Higher Diploma is a well-established pathway.</t>
+          <t>Fact Check: For Secondary 6 students who do not meet the "3322+2" (Degree) or "22222" (HD) HKDSE requirements, the Diploma of Foundation Studies (DFS) and the Diploma of Vocational Education (DVE) are the recognized "Level 3" (Qualifications Framework) pathways. Answer Key Accuracy: Correct. Completion of DFS is widely recognized as equivalent to five Level 2s in the HKDSE for progression to Higher Diploma.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Note that DFS is generally the more common academic foundation for S6 students aiming for IVE Higher Diplomas, whereas DVE often has a stronger focus on specific trades.</t>
+          <t>Ensure the marking scheme accepts "Diploma of Applied Education" (DAE) as well, as it is a common alternative pathway, though DFS/DVE are the specific VTC-branded ones.</t>
         </is>
       </c>
     </row>
@@ -1062,12 +1062,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>VTC maintains over 25 Training Boards and collaborates with industry partners. The benefits listed (internships, equipment, job placement) are the pillars of VTC’s industry collaboration strategy.</t>
+          <t>Fact Check: VTC has over 20 Training Boards and collaborates with thousands of industry partners. Answer Key Accuracy: Correct. The benefits listed (internships/attachments and curriculum relevance) are the primary pillars of their partnership model.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Use the specific VTC terminology "Work-integrated Learning" (WIL) or "Industrial Attachment" for the internship point.</t>
+          <t>Another strong example often cited by VTC is the "Earn &amp; Learn" Scheme, which combines apprenticeship with study. Including this as an example in the marking scheme would be highly relevant.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(notebooks): update execution timestamps and cache results
- Update all notebook execution timestamps to 2026-01-17 19:31:09
- Replace cache misses with cache hits in marking scheme extraction step
- Reduce AI processing time from 316s to 0s through effective caching
- Update verification searcher and formatter to use cached results
- Refresh sample output files with latest execution results
- Improve notebook performance by leveraging agent caching mechanism
</commit_message>
<xml_diff>
--- a/sample/VTC Test Marking Scheme.xlsx
+++ b/sample/VTC Test Marking Scheme.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>This evaluation confirms that the marking scheme is factually accurate and aligns with the official standards and terminology of the Vocational Training Council (VTC) in Hong Kong. Constructive Feedback &amp; Suggestions: 1. Terminology Consistency: The marking scheme uses "Vocational and Professional Education and Training." Ensure that students are not penalized if they use the older term "Vocational Education and Training (VET)," though they should be encouraged to use the full "VPET" for full marks. 2. Grading Guide Clarity: The "General Grading Guide" is repeated multiple times in your document. You only need to state it once at the beginning or end to keep the scheme concise. 3. Qualification Levels: For Q4, it might be helpful to specify that these programmes are at QF Level 3, which allows progression to QF Level 4 (Higher Diploma). This shows a deeper understanding of the Hong Kong Qualifications Framework. Overall Verdict: The marking scheme is highly accurate and ready for use. Citations: [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHdrenv21lbr6yAbKortDcisxfdZFHSlrRnEv9gUneUBMSVzTEWl6XKekV6S7MbYYoBK09-ojdryUxmGGmiHnOT6JaEo-qv000s84W-lBTJiLtDsjGANGt6KzI=), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEiJFve_NPta3q44d6xbREsqbQPsx67t0cZtWXrVYQ-uc6To6BhcKyerxuOSxoHl-fyYG22s-zQIiDHRBqUFnY0_4POv-jjlgvjnf10SgIgasfDZJ5pnrgMXpVXUg==), [vpet.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEIUyTUeZEiL6tNf1Ez8QHkcnLOJ31pG8AqMfDijk_ZMPOwV7wHSzz3caNYHUlQHN3alPkUJVgHLoat43rwokDL0KtVng4iLYIZ2HtJGNVdhYdJM7vylk-U11mBHaLV19h1mOWg3_OdeKZH0aBH), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF1rvYIip6moTtkuw7NtxkC8p66E8wEFQBFHPMsM9pRJShxThnV5fJTc8qoGCMji8JjIbonCwUYOozutyuBmIWoVSqc-98GjUqpHgFu-ER3xtoFoveWyv7RR0od2ve7FuyzTskMeSSKtmr65DQpZyCh20vw1GcXz7z1Idtws6gqDoXhEA==), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF-a-VZrONAx6NwCVnQmgL1op0gzASrbU2LD4tGG6guQEf0PKD7Cks7RvkR1dGbXPyNGxAN2WjhQDDzZlxEz-epBbTLRZuYP-rM9UapMXjKMe6_TTXeWKqikEqWekvatU9Idv2GSsJEHSMCoBc0j_YuAw9i9y4s580M), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFBOG3zXuGfZ38LyLLgWtopL0-u8kKp5sfFkKG04DuH-z3cZoF7MvsxkxzD1SixgIlwx70hmHjkrY06t9WRD30NG_X-qx2Z1MIi9Gpoegfez2BJysy6to2QD1ALDzWxTMvYI4XlIrhYAKCgwQ9uN8e5FXEKCilmHC6usIkOngyjVNQ9)</t>
+          <t>The marking scheme is highly reliable and ready for use. The grading principles are standard and provide clear guidance for examiners. No major factual corrections are required. Citations: [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQElJ6ae_XX1fSF4qAd_yQA0pHnvM38WYAhlD9FcBoidPrMwTnoDHXiVdJU3RfGAN2QFMFtlCtDjSbSIiQTMRe25FfdNaSvLDPsQkR_zLISO6CUQvr8jl4BSpiUu_I3OHLmv0hBS7p5X), [iabhongkong.com](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFPIVY4XTJqLnRvOU3LxfjLPt3iOK6FJ1b__xoGSq88VKE65cFg_K8QKfbS_r35lwrdW3ksMrGw44EDsXMdaYipcWrW7r-5Ogd4_gCuw-LqyUXLTrVufc3Gm5pt8vUqvRfBInA=), [vpet.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFM6tvSdmxdKA3yqUoNlOCR9WBTnj0lsvVHqFe8wU9lqrFTP1fj17oNFPzYXbtwohZDlrcWXJhRLxGEKOhUeNG56R8SPlIUNInrevOwgRKou8XNqqN5HF5B-Cth3TOOUhXf574SDjyuHw==), [ive.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGVPjHvdEClJO6ukbafrBmZPdL9ZeUXyzvHdMZN0_hX5Rhl8AKPbToO6aqdxp-a4UTXIDhggR-EaQc_ZN7g2Mj0HwImZZ3achzmXcAcK1NRLUwd-Yo=), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH0X_eh7ezfDsytvWaPpj3fugqSBmhzHI8Pvh9IBWEZLV2Z2Y_2kqaTFrlkcbEVNj2yi292roCsBLzvO4LjPugEvU4apVaVqP0TY7Fe2QHSM30PJ8H-2-j-4Vf4myspXphg8dqPMEp6LEDhR92EHyMcnaQle84jZAEMO98s1A==), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEuElx1sGvFCohYYBaWDF7ImlaXk0hPbElbF1WLOU3ipgox4NI5CRK5v-tqdkFJOqQoKwCgIXWjGnFbk1UXhYWTRrFboZRsdwxbln1F_HtwWPVTq-NjIrIPqu4h4qPgcceeqkrCOnMKZqDOY9CXUgkpuBvWHA==)</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-01-17 18:59:12</t>
+          <t>2026-01-17 19:31:10</t>
         </is>
       </c>
     </row>
@@ -982,12 +982,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fact Check: VPET does indeed stand for Vocational and Professional Education and Training. The VTC is the statutory body and the largest provider of VPET in Hong Kong. Answer Key Accuracy: Correct. The emphasis on practical skills and workforce development (reducing the skills gap) is the core mission of VPET as defined by the Hong Kong Education Bureau.</t>
+          <t>VPET stands for Vocational and Professional Education and Training. VTC is officially recognized as the largest provider of VPET in Hong Kong, serving approximately 200,000 students annually. The marking points correctly identify the dual focus on practical skills and workforce development.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>You might consider adding a point for mentioning that VPET provides a "parallel pathway" to traditional academic education, as this is a key part of the government's current promotion of the sector.</t>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -1002,12 +1002,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fact Check: IVE (Hong Kong Institute of Vocational Education) is the primary provider of Higher Diploma (HD) and Diploma programmes. THEi (Technological and Higher Education Institute of Hong Kong) was specifically established to offer vocationally-oriented Bachelor’s Degree programmes. Answer Key Accuracy: Correct.</t>
+          <t>IVE is the primary provider of Higher Diplomas (HD), while THEi was established to offer vocationally-oriented Bachelor’s Degrees. The distinction is factually sound.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>To be even more precise, you could mention that THEi degrees are "Applied Degrees," which distinguishes them from traditional research-based degrees at other universities.</t>
+          <t>Consider adding "Top-up Degrees" as a THEi feature for IVE Higher Diploma graduates to highlight the articulation pathway.</t>
         </is>
       </c>
     </row>
@@ -1022,12 +1022,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fact Check: The "Think and Do" approach is the official motto and educational philosophy of the VTC. It is often described in official literature as "hands-on and minds-on." Answer Key Accuracy: Correct. The breakdown of "Think" (theory) and "Do" (practice) is the standard interpretation.</t>
+          <t>VTC’s official motto is "Think and Do," emphasizing the integration of theoretical knowledge with practical application. The marking scheme correctly identifies the synthesis of these elements.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>The marking scheme is solid. You could award bonus marks if a student mentions "problem-solving in real-world contexts," as this is a specific outcome VTC highlights for this approach.</t>
+          <t>Use the term "Applied Learning" in the marking notes, as this is the formal pedagogical term used by the Hong Kong Education Bureau (EDB).</t>
         </is>
       </c>
     </row>
@@ -1042,12 +1042,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fact Check: For Secondary 6 students who do not meet the "3322+2" (Degree) or "22222" (HD) HKDSE requirements, the Diploma of Foundation Studies (DFS) and the Diploma of Vocational Education (DVE) are the recognized "Level 3" (Qualifications Framework) pathways. Answer Key Accuracy: Correct. Completion of DFS is widely recognized as equivalent to five Level 2s in the HKDSE for progression to Higher Diploma.</t>
+          <t>For S6 students not meeting HKDSE requirements, DFS and DVE are the standard VTC entry points. The progression from DFS/DVE to Higher Diploma is a well-established pathway.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ensure the marking scheme accepts "Diploma of Applied Education" (DAE) as well, as it is a common alternative pathway, though DFS/DVE are the specific VTC-branded ones.</t>
+          <t>Note that DFS is generally the more common academic foundation for S6 students aiming for IVE Higher Diplomas, whereas DVE often has a stronger focus on specific trades.</t>
         </is>
       </c>
     </row>
@@ -1062,12 +1062,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fact Check: VTC has over 20 Training Boards and collaborates with thousands of industry partners. Answer Key Accuracy: Correct. The benefits listed (internships/attachments and curriculum relevance) are the primary pillars of their partnership model.</t>
+          <t>VTC maintains over 25 Training Boards and collaborates with industry partners. The benefits listed (internships, equipment, job placement) are the pillars of VTC’s industry collaboration strategy.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Another strong example often cited by VTC is the "Earn &amp; Learn" Scheme, which combines apprenticeship with study. Including this as an example in the marking scheme would be highly relevant.</t>
+          <t>Use the specific VTC terminology "Work-integrated Learning" (WIL) or "Industrial Attachment" for the internship point.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove used code and use markdown libray.
</commit_message>
<xml_diff>
--- a/sample/VTC Test Marking Scheme.xlsx
+++ b/sample/VTC Test Marking Scheme.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>The marking scheme is highly reliable and ready for use. The grading principles are standard and provide clear guidance for examiners. No major factual corrections are required. Citations: [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQElJ6ae_XX1fSF4qAd_yQA0pHnvM38WYAhlD9FcBoidPrMwTnoDHXiVdJU3RfGAN2QFMFtlCtDjSbSIiQTMRe25FfdNaSvLDPsQkR_zLISO6CUQvr8jl4BSpiUu_I3OHLmv0hBS7p5X), [iabhongkong.com](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFPIVY4XTJqLnRvOU3LxfjLPt3iOK6FJ1b__xoGSq88VKE65cFg_K8QKfbS_r35lwrdW3ksMrGw44EDsXMdaYipcWrW7r-5Ogd4_gCuw-LqyUXLTrVufc3Gm5pt8vUqvRfBInA=), [vpet.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFM6tvSdmxdKA3yqUoNlOCR9WBTnj0lsvVHqFe8wU9lqrFTP1fj17oNFPzYXbtwohZDlrcWXJhRLxGEKOhUeNG56R8SPlIUNInrevOwgRKou8XNqqN5HF5B-Cth3TOOUhXf574SDjyuHw==), [ive.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGVPjHvdEClJO6ukbafrBmZPdL9ZeUXyzvHdMZN0_hX5Rhl8AKPbToO6aqdxp-a4UTXIDhggR-EaQc_ZN7g2Mj0HwImZZ3achzmXcAcK1NRLUwd-Yo=), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH0X_eh7ezfDsytvWaPpj3fugqSBmhzHI8Pvh9IBWEZLV2Z2Y_2kqaTFrlkcbEVNj2yi292roCsBLzvO4LjPugEvU4apVaVqP0TY7Fe2QHSM30PJ8H-2-j-4Vf4myspXphg8dqPMEp6LEDhR92EHyMcnaQle84jZAEMO98s1A==), [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEuElx1sGvFCohYYBaWDF7ImlaXk0hPbElbF1WLOU3ipgox4NI5CRK5v-tqdkFJOqQoKwCgIXWjGnFbk1UXhYWTRrFboZRsdwxbln1F_HtwWPVTq-NjIrIPqu4h4qPgcceeqkrCOnMKZqDOY9CXUgkpuBvWHA==)</t>
+          <t>This verification confirms that the marking scheme for the Vocational Training Council (VTC) questions is factually accurate and aligns with the official terminology and educational structure used in Hong Kong. The scheme is ready for use, though formatting could be improved by removing the repeated 'General Grading Guide' after every question. Key references include [vpet.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGmLf3qA-NbRAsCJxLohSy5WUfcUQp3JoX9cvKm4mC89XvOy6kKMWYGa6f1Swx-4Skwz0EHDDAhiEMI_DVP3eikG2pJr-5-0uUyMFGoTmRmgTPUbIuRs032tExj76qbwkEtvHnCwssj0EoM5jbF) and [edb.gov.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHdBIP9v0yD8Fd773H6cMEyA50QrxbI0UFbl0gbxlrf7cioRE4nrFsf0vbsTpObTAzj9SlCZ_LkwIISlI0yvFbShKVQeLUyV9cGF7GgvP3-h7pSNXNTmBe-VuAgLDhcHPZs6Fv7oGBaTSmANEH5Dcv5Biw6nXNEwk_JiuPDfN7EUuS58DMHjiGM2em7dKSEBshh0-6QZN7Age6xpw==).</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-01-17 19:31:10</t>
+          <t>2026-01-17 13:08:42</t>
         </is>
       </c>
     </row>
@@ -982,12 +982,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>VPET stands for Vocational and Professional Education and Training. VTC is officially recognized as the largest provider of VPET in Hong Kong, serving approximately 200,000 students annually. The marking points correctly identify the dual focus on practical skills and workforce development.</t>
+          <t>VPET stands for Vocational and Professional Education and Training. VTC is the largest provider in Hong Kong, focusing on applied knowledge and practical skills to meet industry manpower demands. [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFJYvO9TbDgF9OXxyjr7DNMGr9Qp9vlGWXsbjpYIG9RFp3ufolVwWsOcNI2acQEzX0YJsD_8DTUAKHJnAZjKkZwW7JKk_JXjuD5U1byXuqiF1086GuCEW8_aZPQY_4yHecUjiRgYn9b)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Add a point about 'Multiple Entry and Exit Points' as a reason for VPET's importance, as this is a core part of the VTC's mission to support lifelong learning.</t>
         </is>
       </c>
     </row>
@@ -1002,12 +1002,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>IVE is the primary provider of Higher Diplomas (HD), while THEi was established to offer vocationally-oriented Bachelor’s Degrees. The distinction is factually sound.</t>
+          <t>The distinction is accurate. IVE primarily offers Higher Diplomas (Level 4 on the HK Qualifications Framework), while THEi focuses on applied-science-oriented Bachelor’s Degrees (Level 5). [ive.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHLlQG6t7Rgn5IMd948uiqheJpb_kwy2difShZJiheenw9GgxWrdb7VLuCJzbZTafxjf2Ydgb9u1He5xk8gG-FZkIC1pDoORh0FJS3YuAOUuhiiORD_49YSko5ecROJxzHe0k-NgdGrpsPD-pv7_lqtXg==)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Consider adding "Top-up Degrees" as a THEi feature for IVE Higher Diploma graduates to highlight the articulation pathway.</t>
+          <t>Mention that THEi is part of the government's initiative to develop Universities of Applied Sciences (UAS).</t>
         </is>
       </c>
     </row>
@@ -1022,12 +1022,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>VTC’s official motto is "Think and Do," emphasizing the integration of theoretical knowledge with practical application. The marking scheme correctly identifies the synthesis of these elements.</t>
+          <t>The 'Think and Do' approach is VTC’s signature pedagogy. 'Think' represents theoretical knowledge and 'Do' represents practical application. The requirement for synthesis reflects the applied nature of the curriculum. [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHB-9XYQEOluZAk5_yueLUcBy_HNOfGbOMS02FfP6fWG0YhiytHOr_XEtOPVDFzR7E30i8dLARUgwmfCouI5ImmkcGS8XSDflWxuXCF2zoiYDcEizpbOYlzesZDlBfBTjgTZ9aTNkNKdP-5fhhhtqWcRcnFPHDSqdQF6S37jBC59nQI2OtN)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Use the term "Applied Learning" in the marking notes, as this is the formal pedagogical term used by the Hong Kong Education Bureau (EDB).</t>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -1042,12 +1042,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>For S6 students not meeting HKDSE requirements, DFS and DVE are the standard VTC entry points. The progression from DFS/DVE to Higher Diploma is a well-established pathway.</t>
+          <t>The answer key is correct. The Diploma of Foundation Studies (DFS) is the primary pathway for S6 students, and its completion is recognized as equivalent to Level 2 in five HKDSE subjects. [yc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFcGBeIyA_OzQ9xeLdXKcBAO265Wrw6mGdF46N5KTRlOasxtDByL0PkTcUNxUN9CmGUxeB0QhS5OSjGI6QfyZAMe_cXxWXHxItdcCwkHr19F_-iPehnM4hDgetFSAgXyjSdCy-l6nXsCkcI9HxZKe0=)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Note that DFS is generally the more common academic foundation for S6 students aiming for IVE Higher Diplomas, whereas DVE often has a stronger focus on specific trades.</t>
+          <t>Suggest that students mention the HKQF Level (DFS is Level 3) for extra clarity.</t>
         </is>
       </c>
     </row>
@@ -1062,12 +1062,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>VTC maintains over 25 Training Boards and collaborates with industry partners. The benefits listed (internships, equipment, job placement) are the pillars of VTC’s industry collaboration strategy.</t>
+          <t>The marking scheme is accurate. VTC operates 25 Training Boards to ensure curriculum relevance and provides benefits like Work-Integrated Learning (WIL) and industry-standard equipment. [vtc.edu.hk](https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF3Q9Yjl9SfgsJBJddJZfZXfZAPYHJVDiISr0OiO7wqF-O17oQwyndQnAJrLviPr5EzX_vz_J0IBRQQ2Rx2UKDhbwq_ZXeNkuRpKXqPf-cIXSA6816zUDdLvpaW1K1iHLkFSzWVuWn4AoFklxmP7Q0yy4zvEooYFwn55ibK7iXUic34wA==)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Use the specific VTC terminology "Work-integrated Learning" (WIL) or "Industrial Attachment" for the internship point.</t>
+          <t>Mentioning 'Work-integrated learning' specifically would be a strong addition to the first specific benefit point.</t>
         </is>
       </c>
     </row>

</xml_diff>